<commit_message>
add week 11 basic
</commit_message>
<xml_diff>
--- a/LabX_Advance_10/data/output_report.xlsx
+++ b/LabX_Advance_10/data/output_report.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Audit Log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="SalesData" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Raw Data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SalesData" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Data" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -156,14 +156,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -187,7 +187,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -246,8 +246,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -276,8 +276,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -303,7 +303,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -318,9 +318,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -658,7 +658,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-07T00:37:08.810994</t>
+          <t>2026-10-07T01:02:58.992810</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -685,7 +685,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-07T00:37:08.811973</t>
+          <t>2026-10-07T01:02:58.994117</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -712,7 +712,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-07T00:37:08.812537</t>
+          <t>2026-10-07T01:02:58.994803</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -739,7 +739,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-07T00:37:08.812907</t>
+          <t>2026-10-07T01:02:58.995218</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -766,7 +766,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-07T00:37:08.815531</t>
+          <t>2026-10-07T01:02:58.997989</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -793,7 +793,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-07T00:37:08.815951</t>
+          <t>2026-10-07T01:02:58.998525</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -820,7 +820,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-07T00:37:08.816258</t>
+          <t>2026-10-07T01:02:58.999019</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">

</xml_diff>